<commit_message>
updated measurement reports with dependency correction
</commit_message>
<xml_diff>
--- a/measurements/24/Filled_2D_sections/axial/week24_axial_Batch_Allmarks.xlsx
+++ b/measurements/24/Filled_2D_sections/axial/week24_axial_Batch_Allmarks.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:X27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,12 +487,57 @@
           <t>mean_depth_mm</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Primary_count</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Primary_v1_mm</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary_count</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary_v1_mm</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary_v2_mm</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary_v3_mm</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Tertiary_count</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Tertiary_v1_mm</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Unclassified_count</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Mean</t>
         </is>
@@ -506,43 +551,67 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5.537180249851279</v>
+        <v>2110.657596371882</v>
       </c>
       <c r="D2" t="n">
-        <v>13.76828198898129</v>
+        <v>268.8093150229681</v>
       </c>
       <c r="E2" t="n">
-        <v>9.853412104815972</v>
+        <v>192.3761410940261</v>
       </c>
       <c r="F2" t="n">
         <v>1.397311088029281</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3670616569789488</v>
+        <v>0.3670616569789486</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I2" t="n">
-        <v>1.365853658536585</v>
+        <v>3.184523809523809</v>
       </c>
       <c r="J2" t="n">
-        <v>1.365853658536585</v>
+        <v>26.66666666666666</v>
       </c>
       <c r="K2" t="n">
-        <v>1.365853658536585</v>
-      </c>
-      <c r="N2" t="inlineStr">
+        <v>9.475911458333332</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>26.66666666666666</v>
+      </c>
+      <c r="N2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O2" t="n">
+        <v>4.388020833333333</v>
+      </c>
+      <c r="P2" t="n">
+        <v>3.664434523809524</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>3.184523809523809</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="inlineStr">
         <is>
           <t>area</t>
         </is>
       </c>
-      <c r="O2" s="2" t="n">
-        <v>5.487314098750744</v>
+      <c r="X2" s="2" t="n">
+        <v>2091.649659863945</v>
       </c>
     </row>
     <row r="3">
@@ -553,17 +622,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5.634146341463415</v>
+        <v>2147.619047619047</v>
       </c>
       <c r="D3" t="n">
-        <v>13.58989887121247</v>
+        <v>265.3265970093863</v>
       </c>
       <c r="E3" t="n">
-        <v>9.930767495457719</v>
+        <v>193.8864130065554</v>
       </c>
       <c r="F3" t="n">
         <v>1.368464106870735</v>
@@ -572,24 +641,48 @@
         <v>0.3833588885776882</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>1.274771341463415</v>
+        <v>3.61235119047619</v>
       </c>
       <c r="J3" t="n">
-        <v>1.274771341463415</v>
+        <v>24.88839285714285</v>
       </c>
       <c r="K3" t="n">
-        <v>1.274771341463415</v>
-      </c>
-      <c r="N3" t="inlineStr">
+        <v>9.176432291666666</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>24.88839285714285</v>
+      </c>
+      <c r="N3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4.358258928571428</v>
+      </c>
+      <c r="P3" t="n">
+        <v>3.84672619047619</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>3.61235119047619</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>perimeter</t>
         </is>
       </c>
-      <c r="O3" s="2" t="n">
-        <v>11.60130994130926</v>
+      <c r="X3" s="2" t="n">
+        <v>226.5017655207997</v>
       </c>
     </row>
     <row r="4">
@@ -600,17 +693,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5.684711481261155</v>
+        <v>2166.893424036281</v>
       </c>
       <c r="D4" t="n">
-        <v>13.50907671742323</v>
+        <v>263.7486406735011</v>
       </c>
       <c r="E4" t="n">
-        <v>9.959342462260549</v>
+        <v>194.4443052155631</v>
       </c>
       <c r="F4" t="n">
         <v>1.356422551851578</v>
@@ -619,24 +712,48 @@
         <v>0.3914415798912779</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>1.268292682926829</v>
+        <v>3.647693452380952</v>
       </c>
       <c r="J4" t="n">
-        <v>1.268292682926829</v>
+        <v>24.76190476190476</v>
       </c>
       <c r="K4" t="n">
-        <v>1.268292682926829</v>
-      </c>
-      <c r="N4" t="inlineStr">
+        <v>9.36337425595238</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>24.76190476190476</v>
+      </c>
+      <c r="N4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" t="n">
+        <v>4.640997023809524</v>
+      </c>
+      <c r="P4" t="n">
+        <v>4.402901785714286</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>3.647693452380952</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>perimeter_convex</t>
         </is>
       </c>
-      <c r="O4" s="2" t="n">
-        <v>9.788889244707621</v>
+      <c r="X4" s="2" t="n">
+        <v>191.1164090633392</v>
       </c>
     </row>
     <row r="5">
@@ -647,42 +764,66 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5.687983343248067</v>
+        <v>2168.140589569161</v>
       </c>
       <c r="D5" t="n">
-        <v>13.47458366940661</v>
+        <v>263.0752049741291</v>
       </c>
       <c r="E5" t="n">
-        <v>10.00812293552771</v>
+        <v>195.3966858841124</v>
       </c>
       <c r="F5" t="n">
-        <v>1.346364723556039</v>
+        <v>1.346364723556038</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3936746672037672</v>
+        <v>0.3936746672037674</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I5" t="n">
-        <v>1.24390243902439</v>
+        <v>3.809523809523809</v>
       </c>
       <c r="J5" t="n">
-        <v>1.24390243902439</v>
+        <v>24.28571428571428</v>
       </c>
       <c r="K5" t="n">
-        <v>1.24390243902439</v>
-      </c>
-      <c r="N5" t="inlineStr">
+        <v>9.315941220238095</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4.953497023809524</v>
+      </c>
+      <c r="P5" t="n">
+        <v>4.215029761904762</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>3.809523809523809</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="inlineStr">
         <is>
           <t>LGI</t>
         </is>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="X5" s="2" t="n">
         <v>1.182492333946165</v>
       </c>
     </row>
@@ -694,42 +835,66 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.684414039262344</v>
+        <v>2166.780045351474</v>
       </c>
       <c r="D6" t="n">
-        <v>13.45437815131211</v>
+        <v>262.6807162875221</v>
       </c>
       <c r="E6" t="n">
-        <v>10.09139644808886</v>
+        <v>197.0225020817348</v>
       </c>
       <c r="F6" t="n">
         <v>1.333252362101</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3946102007415216</v>
+        <v>0.3946102007415215</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I6" t="n">
-        <v>1.24390243902439</v>
+        <v>4.285714285714286</v>
       </c>
       <c r="J6" t="n">
-        <v>1.24390243902439</v>
+        <v>24.28571428571428</v>
       </c>
       <c r="K6" t="n">
-        <v>1.24390243902439</v>
-      </c>
-      <c r="N6" t="inlineStr">
+        <v>9.658668154761905</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="N6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" t="n">
+        <v>5.176711309523809</v>
+      </c>
+      <c r="P6" t="n">
+        <v>4.886532738095238</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="inlineStr">
         <is>
           <t>Compactness</t>
         </is>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="X6" s="2" t="n">
         <v>0.5355695581830604</v>
       </c>
     </row>
@@ -741,43 +906,67 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5.677275431290899</v>
+        <v>2164.0589569161</v>
       </c>
       <c r="D7" t="n">
-        <v>13.3164060900851</v>
+        <v>259.9869760445186</v>
       </c>
       <c r="E7" t="n">
-        <v>10.05690344077785</v>
+        <v>196.3490671770913</v>
       </c>
       <c r="F7" t="n">
         <v>1.324105990328087</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4023238392977693</v>
+        <v>0.4023238392977692</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I7" t="n">
-        <v>1.219512195121951</v>
+        <v>4.572172619047619</v>
       </c>
       <c r="J7" t="n">
-        <v>1.219512195121951</v>
+        <v>23.80952380952381</v>
       </c>
       <c r="K7" t="n">
-        <v>1.219512195121951</v>
-      </c>
-      <c r="N7" t="inlineStr">
+        <v>9.631696428571429</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>23.80952380952381</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" t="n">
+        <v>5.128348214285714</v>
+      </c>
+      <c r="P7" t="n">
+        <v>5.016741071428571</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>4.572172619047619</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="inlineStr">
         <is>
           <t>Sulci_count</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n">
-        <v>0.7</v>
+      <c r="X7" s="2" t="n">
+        <v>3.8</v>
       </c>
     </row>
     <row r="8">
@@ -788,43 +977,67 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5.673111243307555</v>
+        <v>2162.471655328798</v>
       </c>
       <c r="D8" t="n">
-        <v>13.01188704734895</v>
+        <v>254.0416042577652</v>
       </c>
       <c r="E8" t="n">
-        <v>10.08547839885805</v>
+        <v>196.9069592158</v>
       </c>
       <c r="F8" t="n">
         <v>1.290160618342334</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4210664069714485</v>
+        <v>0.4210664069714486</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I8" t="n">
-        <v>1.142149390243902</v>
+        <v>4.600074404761904</v>
       </c>
       <c r="J8" t="n">
-        <v>1.142149390243902</v>
+        <v>22.29910714285714</v>
       </c>
       <c r="K8" t="n">
-        <v>1.142149390243902</v>
-      </c>
-      <c r="N8" t="inlineStr">
+        <v>9.32524181547619</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>22.29910714285714</v>
+      </c>
+      <c r="N8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" t="n">
+        <v>5.433407738095238</v>
+      </c>
+      <c r="P8" t="n">
+        <v>4.968377976190476</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>4.600074404761904</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="inlineStr">
         <is>
           <t>min_depth_mm</t>
         </is>
       </c>
-      <c r="O8" s="2" t="n">
-        <v>1.004600391986063</v>
+      <c r="X8" s="2" t="n">
+        <v>3.521763392857142</v>
       </c>
     </row>
     <row r="9">
@@ -835,17 +1048,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5.656751933372993</v>
+        <v>2156.235827664399</v>
       </c>
       <c r="D9" t="n">
-        <v>12.36488920886342</v>
+        <v>241.4097416968573</v>
       </c>
       <c r="E9" t="n">
-        <v>9.996286828343461</v>
+        <v>195.1655999819438</v>
       </c>
       <c r="F9" t="n">
         <v>1.236948220993822</v>
@@ -854,24 +1067,48 @@
         <v>0.4649396017004886</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>1.04639862804878</v>
+        <v>4.123883928571428</v>
       </c>
       <c r="J9" t="n">
-        <v>1.04639862804878</v>
+        <v>20.4296875</v>
       </c>
       <c r="K9" t="n">
-        <v>1.04639862804878</v>
-      </c>
-      <c r="N9" t="inlineStr">
+        <v>8.704892113095239</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20.4296875</v>
+      </c>
+      <c r="N9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" t="n">
+        <v>5.431547619047619</v>
+      </c>
+      <c r="P9" t="n">
+        <v>4.834449404761904</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>4.123883928571428</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="inlineStr">
         <is>
           <t>max_depth_mm</t>
         </is>
       </c>
-      <c r="O9" s="2" t="n">
-        <v>1.004600391986063</v>
+      <c r="X9" s="2" t="n">
+        <v>16.25306919642857</v>
       </c>
     </row>
     <row r="10">
@@ -882,43 +1119,67 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5.591314693634741</v>
+        <v>2131.292517006802</v>
       </c>
       <c r="D10" t="n">
-        <v>11.74748169503561</v>
+        <v>229.3555949983142</v>
       </c>
       <c r="E10" t="n">
-        <v>9.996286837066092</v>
+        <v>195.1656001522427</v>
       </c>
       <c r="F10" t="n">
         <v>1.175184534669024</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5091365158295331</v>
+        <v>0.5091365158295332</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>0.9184451219512195</v>
+        <v>4.123883928571428</v>
       </c>
       <c r="J10" t="n">
-        <v>0.9184451219512195</v>
+        <v>17.93154761904762</v>
       </c>
       <c r="K10" t="n">
-        <v>0.9184451219512195</v>
-      </c>
-      <c r="N10" t="inlineStr">
+        <v>8.043154761904761</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>17.93154761904762</v>
+      </c>
+      <c r="N10" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" t="n">
+        <v>5.954241071428571</v>
+      </c>
+      <c r="P10" t="n">
+        <v>4.162946428571428</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>4.123883928571428</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="inlineStr">
         <is>
           <t>mean_depth_mm</t>
         </is>
       </c>
-      <c r="O10" s="2" t="n">
-        <v>1.004600391986063</v>
+      <c r="X10" s="2" t="n">
+        <v>7.37939453125</v>
       </c>
     </row>
     <row r="11">
@@ -929,35 +1190,67 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5.542534205829863</v>
+        <v>2112.698412698413</v>
       </c>
       <c r="D11" t="n">
-        <v>11.59277082361826</v>
+        <v>226.3350494134994</v>
       </c>
       <c r="E11" t="n">
-        <v>9.976081307341413</v>
+        <v>194.7711112385704</v>
       </c>
       <c r="F11" t="n">
         <v>1.162056569756215</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5182552917323634</v>
+        <v>0.5182552917323635</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I11" t="n">
-        <v>0.9152057926829269</v>
+        <v>3.655133928571428</v>
       </c>
       <c r="J11" t="n">
-        <v>0.9152057926829269</v>
+        <v>17.86830357142857</v>
       </c>
       <c r="K11" t="n">
-        <v>0.9152057926829269</v>
+        <v>7.792503720238094</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>17.86830357142857</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" t="n">
+        <v>5.613839285714286</v>
+      </c>
+      <c r="P11" t="n">
+        <v>4.032738095238095</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>3.655133928571428</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Primary_count</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="n">
+        <v>0.95</v>
       </c>
     </row>
     <row r="12">
@@ -968,35 +1261,67 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5.43575252825699</v>
+        <v>2071.995464852608</v>
       </c>
       <c r="D12" t="n">
-        <v>10.9527064038486</v>
+        <v>213.8385535989489</v>
       </c>
       <c r="E12" t="n">
-        <v>9.961793829755086</v>
+        <v>194.4921652475993</v>
       </c>
       <c r="F12" t="n">
         <v>1.099471299148326</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5694120429215982</v>
+        <v>0.5694120429215983</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6746379573170732</v>
+        <v>3.809523809523809</v>
       </c>
       <c r="J12" t="n">
-        <v>0.6746379573170732</v>
+        <v>13.17150297619048</v>
       </c>
       <c r="K12" t="n">
-        <v>0.6746379573170732</v>
+        <v>6.821521577380953</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>13.17150297619048</v>
+      </c>
+      <c r="N12" t="n">
+        <v>3</v>
+      </c>
+      <c r="O12" t="n">
+        <v>5.887276785714286</v>
+      </c>
+      <c r="P12" t="n">
+        <v>4.417782738095238</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>3.809523809523809</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Primary_v1_mm</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="n">
+        <v>16.71659617794486</v>
       </c>
     </row>
     <row r="13">
@@ -1007,17 +1332,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5.391433670434266</v>
+        <v>2055.102040816326</v>
       </c>
       <c r="D13" t="n">
-        <v>10.90984398271979</v>
+        <v>213.0017158531007</v>
       </c>
       <c r="E13" t="n">
-        <v>9.967711890616068</v>
+        <v>194.6077083405994</v>
       </c>
       <c r="F13" t="n">
         <v>1.094518391225842</v>
@@ -1026,16 +1351,48 @@
         <v>0.5692159365031623</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6722560975609756</v>
+        <v>4.285714285714286</v>
       </c>
       <c r="J13" t="n">
-        <v>0.6722560975609756</v>
+        <v>13.125</v>
       </c>
       <c r="K13" t="n">
-        <v>0.6722560975609756</v>
+        <v>6.938709077380952</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>13.125</v>
+      </c>
+      <c r="N13" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" t="n">
+        <v>5.846354166666666</v>
+      </c>
+      <c r="P13" t="n">
+        <v>4.497767857142857</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Secondary_count</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="n">
+        <v>2.7</v>
       </c>
     </row>
     <row r="14">
@@ -1046,35 +1403,67 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5.322724568709102</v>
+        <v>2028.91156462585</v>
       </c>
       <c r="D14" t="n">
-        <v>10.5994068413246</v>
+        <v>206.940800235385</v>
       </c>
       <c r="E14" t="n">
-        <v>9.817903672776572</v>
+        <v>191.6828812303997</v>
       </c>
       <c r="F14" t="n">
         <v>1.079599799977159</v>
       </c>
       <c r="G14" t="n">
-        <v>0.5953614813833233</v>
+        <v>0.5953614813833235</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I14" t="n">
-        <v>0.5525914634146342</v>
+        <v>4.326636904761904</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5525914634146342</v>
+        <v>10.78869047619048</v>
       </c>
       <c r="K14" t="n">
-        <v>0.5525914634146342</v>
+        <v>6.392764136904762</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>10.78869047619048</v>
+      </c>
+      <c r="N14" t="n">
+        <v>3</v>
+      </c>
+      <c r="O14" t="n">
+        <v>5.693824404761904</v>
+      </c>
+      <c r="P14" t="n">
+        <v>4.761904761904762</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>4.326636904761904</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Secondary_v1_mm</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="n">
+        <v>5.279668898809524</v>
       </c>
     </row>
     <row r="15">
@@ -1085,17 +1474,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5.310232004759072</v>
+        <v>2024.149659863945</v>
       </c>
       <c r="D15" t="n">
-        <v>10.59103744495206</v>
+        <v>206.7773977347782</v>
       </c>
       <c r="E15" t="n">
-        <v>9.823821745267729</v>
+        <v>191.7984245504652</v>
       </c>
       <c r="F15" t="n">
         <v>1.078097477700459</v>
@@ -1104,16 +1493,48 @@
         <v>0.5949032655949343</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I15" t="n">
-        <v>0.5264862804878049</v>
+        <v>4.322916666666666</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5264862804878049</v>
+        <v>10.27901785714286</v>
       </c>
       <c r="K15" t="n">
-        <v>0.5264862804878049</v>
+        <v>6.395089285714285</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>10.27901785714286</v>
+      </c>
+      <c r="N15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" t="n">
+        <v>5.74032738095238</v>
+      </c>
+      <c r="P15" t="n">
+        <v>5.238095238095238</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>4.322916666666666</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Secondary_v2_mm</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="n">
+        <v>4.428258145363408</v>
       </c>
     </row>
     <row r="16">
@@ -1124,26 +1545,67 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5.309637120761452</v>
+        <v>2023.922902494331</v>
       </c>
       <c r="D16" t="n">
-        <v>10.28651838477065</v>
+        <v>200.8320256074269</v>
       </c>
       <c r="E16" t="n">
-        <v>9.679931640625</v>
+        <v>188.9891415550595</v>
       </c>
       <c r="F16" t="n">
-        <v>1.062664362380403</v>
+        <v>1.062664362380402</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6305766597282488</v>
+        <v>0.6305766597282489</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2.96875</v>
+      </c>
+      <c r="J16" t="n">
+        <v>9.523809523809524</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5.809616815476191</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>9.523809523809524</v>
+      </c>
+      <c r="N16" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" t="n">
+        <v>5.5078125</v>
+      </c>
+      <c r="P16" t="n">
+        <v>5.238095238095238</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>2.96875</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Secondary_v3_mm</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="n">
+        <v>3.955233134920634</v>
       </c>
     </row>
     <row r="17">
@@ -1154,17 +1616,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5.334324806662701</v>
+        <v>2033.333333333333</v>
       </c>
       <c r="D17" t="n">
-        <v>10.07710898504025</v>
+        <v>196.7435563745953</v>
       </c>
       <c r="E17" t="n">
-        <v>9.596658148416658</v>
+        <v>187.3633257548014</v>
       </c>
       <c r="F17" t="n">
         <v>1.050064390040074</v>
@@ -1173,7 +1635,48 @@
         <v>0.6601116679429371</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1.741071428571428</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8.833705357142856</v>
+      </c>
+      <c r="K17" t="n">
+        <v>5.110677083333332</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>8.833705357142856</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>5.267857142857142</v>
+      </c>
+      <c r="P17" t="n">
+        <v>4.600074404761904</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1.741071428571428</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Tertiary_count</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="18">
@@ -1184,17 +1687,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5.351279000594884</v>
+        <v>2039.795918367347</v>
       </c>
       <c r="D18" t="n">
-        <v>9.876068926439054</v>
+        <v>192.8184885638101</v>
       </c>
       <c r="E18" t="n">
-        <v>9.430111120386822</v>
+        <v>184.1116933027903</v>
       </c>
       <c r="F18" t="n">
         <v>1.047290832563799</v>
@@ -1203,7 +1706,45 @@
         <v>0.6894443770362386</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4.135044642857142</v>
+      </c>
+      <c r="J18" t="n">
+        <v>8.095238095238095</v>
+      </c>
+      <c r="K18" t="n">
+        <v>5.505332341269841</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>8.095238095238095</v>
+      </c>
+      <c r="N18" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="P18" t="n">
+        <v>4.135044642857142</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Tertiary_v1_mm</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="n">
+        <v>1.348586309523809</v>
       </c>
     </row>
     <row r="19">
@@ -1214,17 +1755,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.348304580606782</v>
+        <v>2038.662131519274</v>
       </c>
       <c r="D19" t="n">
-        <v>9.807082917632126</v>
+        <v>191.4716188680558</v>
       </c>
       <c r="E19" t="n">
-        <v>9.340919558594868</v>
+        <v>182.3703342392331</v>
       </c>
       <c r="F19" t="n">
         <v>1.049905510492094</v>
@@ -1233,6 +1774,44 @@
         <v>0.6987893887455956</v>
       </c>
       <c r="H19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2.925967261904762</v>
+      </c>
+      <c r="J19" t="n">
+        <v>8.376116071428571</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5.19593253968254</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>8.376116071428571</v>
+      </c>
+      <c r="N19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="P19" t="n">
+        <v>2.925967261904762</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Unclassified_count</t>
+        </is>
+      </c>
+      <c r="X19" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1244,17 +1823,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5.323616894705533</v>
+        <v>2029.251700680272</v>
       </c>
       <c r="D20" t="n">
-        <v>9.663192827527116</v>
+        <v>188.6623361564818</v>
       </c>
       <c r="E20" t="n">
-        <v>9.202947514813122</v>
+        <v>179.6765943368276</v>
       </c>
       <c r="F20" t="n">
         <v>1.050010641913711</v>
@@ -1263,6 +1842,36 @@
         <v>0.7164326452392196</v>
       </c>
       <c r="H20" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1.329985119047619</v>
+      </c>
+      <c r="J20" t="n">
+        <v>8.195684523809524</v>
+      </c>
+      <c r="K20" t="n">
+        <v>4.693080357142857</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>8.195684523809524</v>
+      </c>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>4.553571428571428</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="n">
+        <v>1.329985119047619</v>
+      </c>
+      <c r="T20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1274,17 +1883,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>not_full_slice</t>
+          <t>axial</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5.249553837001785</v>
+        <v>2001.020408163265</v>
       </c>
       <c r="D21" t="n">
-        <v>9.433577848643791</v>
+        <v>184.1793770449502</v>
       </c>
       <c r="E21" t="n">
-        <v>9.0019075143628</v>
+        <v>175.751527661369</v>
       </c>
       <c r="F21" t="n">
         <v>1.047953206983325</v>
@@ -1293,6 +1902,36 @@
         <v>0.7412750496411439</v>
       </c>
       <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.9747023809523809</v>
+      </c>
+      <c r="J21" t="n">
+        <v>7.446056547619047</v>
+      </c>
+      <c r="K21" t="n">
+        <v>4.237351190476191</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>2</v>
+      </c>
+      <c r="O21" t="n">
+        <v>7.446056547619047</v>
+      </c>
+      <c r="P21" t="n">
+        <v>4.291294642857142</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.9747023809523809</v>
+      </c>
+      <c r="T21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1303,7 +1942,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.02439024390243903</v>
+        <v>0.4761904761904762</v>
       </c>
     </row>
     <row r="23">
@@ -1326,6 +1965,38 @@
       </c>
       <c r="B24" t="n">
         <v>25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ScalebarMeasuredPixels:</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ScalebarRealWorldLength:</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ScalebarRealWorldUnit:</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>